<commit_message>
직업별 Card 추가와 Title -> Collection 연결
직업별 카드 추가 및 Title -> Collector 연결
</commit_message>
<xml_diff>
--- a/ProjectC/Assets/Excel/CardData.xlsx
+++ b/ProjectC/Assets/Excel/CardData.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="284">
   <si>
     <t>Name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -876,6 +876,316 @@
   </si>
   <si>
     <t>비전</t>
+  </si>
+  <si>
+    <t>마법사</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Arcane_Missiles</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mirror_Image</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Arcane_Explosion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Frostbolt</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Magic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Arcane_Intellect</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Frost_Nova</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Original</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fireball</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Polymorph</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Water_Elemental</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>정령</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Flamestrike</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Blessing_of_Might</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>성기사</t>
+  </si>
+  <si>
+    <t>Hand_of_Protection</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Humility</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Light's_Justice</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Holy_Light</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Blessing_of_Kings</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Consecration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hammer_of_Wrath</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Truesilver_Champion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Guardian_of_Kings</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Holy_Smite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>사제</t>
+  </si>
+  <si>
+    <t>Mind_Vision</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Power_Word-_Shield</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shadow_Word-_Pain</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shadow_Word-_Death</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Holy_Nova</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>None</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mind_Control</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Backstab</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>도적</t>
+  </si>
+  <si>
+    <t>Deadly_Poison</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sinister_Strike</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sap</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fan_of_Knives</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assassin's_Blade</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assassinate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sprint</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ancestral_Healing</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>주술사</t>
+  </si>
+  <si>
+    <t>Totemic_Might</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Frost_Shock</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rockbiter_Weapon</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Flametongue_Totem</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Minion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Windfury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Windspeaker</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bloodlust</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>주술사</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fire_Elemental</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sacrificial_Pact</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>흑마법사</t>
+  </si>
+  <si>
+    <t>Soulfire</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Corruption</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mortal_Coil</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Voidwalker</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Felstalker</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Drain_Life</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shadow_Bolt</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hellfire</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dread_Infernal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Execute</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전사</t>
+  </si>
+  <si>
+    <t>전사</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Whirlwind</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cleave</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fiery_War_Axe</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Heroic_Strike</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Charge</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shield_Block</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Warsong_Commander</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kor'kron_Elite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Arcanite_Reaper</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1214,7 +1524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q64"/>
+  <dimension ref="A1:Q129"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.875" customWidth="1"/>
@@ -3573,6 +3883,1534 @@
         <v>199</v>
       </c>
     </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
+        <v>63</v>
+      </c>
+      <c r="C65">
+        <v>1</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H65" t="s">
+        <v>40</v>
+      </c>
+      <c r="I65" t="s">
+        <v>9</v>
+      </c>
+      <c r="J65" t="s">
+        <v>205</v>
+      </c>
+      <c r="K65" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
+        <v>64</v>
+      </c>
+      <c r="C66">
+        <v>1</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="H66" t="s">
+        <v>40</v>
+      </c>
+      <c r="I66" t="s">
+        <v>210</v>
+      </c>
+      <c r="J66" t="s">
+        <v>205</v>
+      </c>
+      <c r="K66" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
+        <v>65</v>
+      </c>
+      <c r="C67">
+        <v>2</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H67" t="s">
+        <v>40</v>
+      </c>
+      <c r="I67" t="s">
+        <v>9</v>
+      </c>
+      <c r="J67" t="s">
+        <v>205</v>
+      </c>
+      <c r="K67" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A68" s="1">
+        <v>66</v>
+      </c>
+      <c r="C68">
+        <v>2</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="H68" t="s">
+        <v>40</v>
+      </c>
+      <c r="I68" t="s">
+        <v>9</v>
+      </c>
+      <c r="J68" t="s">
+        <v>205</v>
+      </c>
+      <c r="K68" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A69" s="1">
+        <v>67</v>
+      </c>
+      <c r="C69">
+        <v>3</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="H69" t="s">
+        <v>40</v>
+      </c>
+      <c r="I69" t="s">
+        <v>9</v>
+      </c>
+      <c r="J69" t="s">
+        <v>205</v>
+      </c>
+      <c r="K69" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A70" s="1">
+        <v>68</v>
+      </c>
+      <c r="C70">
+        <v>3</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="H70" t="s">
+        <v>40</v>
+      </c>
+      <c r="I70" t="s">
+        <v>9</v>
+      </c>
+      <c r="J70" t="s">
+        <v>205</v>
+      </c>
+      <c r="K70" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A71" s="1">
+        <v>69</v>
+      </c>
+      <c r="C71">
+        <v>4</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="H71" t="s">
+        <v>40</v>
+      </c>
+      <c r="I71" t="s">
+        <v>9</v>
+      </c>
+      <c r="J71" t="s">
+        <v>205</v>
+      </c>
+      <c r="K71" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A72" s="1">
+        <v>70</v>
+      </c>
+      <c r="C72">
+        <v>4</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="H72" t="s">
+        <v>40</v>
+      </c>
+      <c r="I72" t="s">
+        <v>9</v>
+      </c>
+      <c r="J72" t="s">
+        <v>205</v>
+      </c>
+      <c r="K72" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A73" s="1">
+        <v>71</v>
+      </c>
+      <c r="C73">
+        <v>4</v>
+      </c>
+      <c r="D73">
+        <v>3</v>
+      </c>
+      <c r="E73">
+        <v>6</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H73" t="s">
+        <v>40</v>
+      </c>
+      <c r="I73" t="s">
+        <v>8</v>
+      </c>
+      <c r="J73" t="s">
+        <v>205</v>
+      </c>
+      <c r="K73" t="s">
+        <v>15</v>
+      </c>
+      <c r="L73" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A74" s="1">
+        <v>72</v>
+      </c>
+      <c r="C74">
+        <v>7</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="H74" t="s">
+        <v>40</v>
+      </c>
+      <c r="I74" t="s">
+        <v>9</v>
+      </c>
+      <c r="J74" t="s">
+        <v>205</v>
+      </c>
+      <c r="K74" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A75" s="1">
+        <v>73</v>
+      </c>
+      <c r="C75">
+        <v>1</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="H75" t="s">
+        <v>40</v>
+      </c>
+      <c r="I75" t="s">
+        <v>9</v>
+      </c>
+      <c r="J75" t="s">
+        <v>220</v>
+      </c>
+      <c r="K75" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A76" s="1">
+        <v>74</v>
+      </c>
+      <c r="C76">
+        <v>1</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="H76" t="s">
+        <v>40</v>
+      </c>
+      <c r="I76" t="s">
+        <v>9</v>
+      </c>
+      <c r="J76" t="s">
+        <v>220</v>
+      </c>
+      <c r="K76" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A77" s="1">
+        <v>75</v>
+      </c>
+      <c r="C77">
+        <v>1</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="H77" t="s">
+        <v>40</v>
+      </c>
+      <c r="I77" t="s">
+        <v>9</v>
+      </c>
+      <c r="J77" t="s">
+        <v>220</v>
+      </c>
+      <c r="K77" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A78" s="1">
+        <v>76</v>
+      </c>
+      <c r="C78">
+        <v>1</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H78" t="s">
+        <v>40</v>
+      </c>
+      <c r="J78" t="s">
+        <v>220</v>
+      </c>
+      <c r="K78" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A79" s="1">
+        <v>77</v>
+      </c>
+      <c r="C79">
+        <v>2</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="H79" t="s">
+        <v>40</v>
+      </c>
+      <c r="I79" t="s">
+        <v>9</v>
+      </c>
+      <c r="J79" t="s">
+        <v>220</v>
+      </c>
+      <c r="K79" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A80" s="1">
+        <v>78</v>
+      </c>
+      <c r="C80">
+        <v>4</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="H80" t="s">
+        <v>40</v>
+      </c>
+      <c r="I80" t="s">
+        <v>210</v>
+      </c>
+      <c r="J80" t="s">
+        <v>220</v>
+      </c>
+      <c r="K80" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A81" s="1">
+        <v>79</v>
+      </c>
+      <c r="C81">
+        <v>4</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="H81" t="s">
+        <v>40</v>
+      </c>
+      <c r="I81" t="s">
+        <v>210</v>
+      </c>
+      <c r="J81" t="s">
+        <v>220</v>
+      </c>
+      <c r="K81" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A82" s="1">
+        <v>80</v>
+      </c>
+      <c r="C82">
+        <v>4</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="H82" t="s">
+        <v>40</v>
+      </c>
+      <c r="I82" t="s">
+        <v>9</v>
+      </c>
+      <c r="J82" t="s">
+        <v>220</v>
+      </c>
+      <c r="K82" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A83" s="1">
+        <v>81</v>
+      </c>
+      <c r="C83">
+        <v>4</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="H83" t="s">
+        <v>40</v>
+      </c>
+      <c r="J83" t="s">
+        <v>220</v>
+      </c>
+      <c r="K83" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A84" s="1">
+        <v>82</v>
+      </c>
+      <c r="C84">
+        <v>7</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="H84" t="s">
+        <v>40</v>
+      </c>
+      <c r="I84" t="s">
+        <v>8</v>
+      </c>
+      <c r="J84" t="s">
+        <v>220</v>
+      </c>
+      <c r="K84" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A85" s="1">
+        <v>83</v>
+      </c>
+      <c r="C85">
+        <v>1</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="H85" t="s">
+        <v>40</v>
+      </c>
+      <c r="I85" t="s">
+        <v>9</v>
+      </c>
+      <c r="J85" t="s">
+        <v>231</v>
+      </c>
+      <c r="K85" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A86" s="1">
+        <v>84</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H86" t="s">
+        <v>40</v>
+      </c>
+      <c r="I86" t="s">
+        <v>210</v>
+      </c>
+      <c r="J86" t="s">
+        <v>231</v>
+      </c>
+      <c r="K86" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A87" s="1">
+        <v>85</v>
+      </c>
+      <c r="C87">
+        <v>1</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="H87" t="s">
+        <v>40</v>
+      </c>
+      <c r="I87" t="s">
+        <v>210</v>
+      </c>
+      <c r="J87" t="s">
+        <v>231</v>
+      </c>
+      <c r="K87" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A88" s="1">
+        <v>86</v>
+      </c>
+      <c r="C88">
+        <v>2</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="H88" t="s">
+        <v>237</v>
+      </c>
+      <c r="I88" t="s">
+        <v>9</v>
+      </c>
+      <c r="J88" t="s">
+        <v>231</v>
+      </c>
+      <c r="K88" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A89" s="1">
+        <v>87</v>
+      </c>
+      <c r="C89">
+        <v>3</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="H89" t="s">
+        <v>40</v>
+      </c>
+      <c r="I89" t="s">
+        <v>9</v>
+      </c>
+      <c r="J89" t="s">
+        <v>231</v>
+      </c>
+      <c r="K89" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A90" s="1">
+        <v>88</v>
+      </c>
+      <c r="C90">
+        <v>5</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="H90" t="s">
+        <v>40</v>
+      </c>
+      <c r="I90" t="s">
+        <v>9</v>
+      </c>
+      <c r="J90" t="s">
+        <v>231</v>
+      </c>
+      <c r="K90" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A91" s="1">
+        <v>89</v>
+      </c>
+      <c r="C91">
+        <v>10</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="H91" t="s">
+        <v>40</v>
+      </c>
+      <c r="I91" t="s">
+        <v>9</v>
+      </c>
+      <c r="J91" t="s">
+        <v>231</v>
+      </c>
+      <c r="K91" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A92" s="1">
+        <v>90</v>
+      </c>
+      <c r="C92">
+        <v>0</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="H92" t="s">
+        <v>40</v>
+      </c>
+      <c r="I92" t="s">
+        <v>9</v>
+      </c>
+      <c r="J92" t="s">
+        <v>240</v>
+      </c>
+      <c r="K92" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A93" s="1">
+        <v>91</v>
+      </c>
+      <c r="C93">
+        <v>1</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="H93" t="s">
+        <v>40</v>
+      </c>
+      <c r="I93" t="s">
+        <v>9</v>
+      </c>
+      <c r="J93" t="s">
+        <v>240</v>
+      </c>
+      <c r="K93" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A94" s="1">
+        <v>92</v>
+      </c>
+      <c r="C94">
+        <v>1</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="H94" t="s">
+        <v>40</v>
+      </c>
+      <c r="I94" t="s">
+        <v>210</v>
+      </c>
+      <c r="J94" t="s">
+        <v>240</v>
+      </c>
+      <c r="K94" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A95" s="1">
+        <v>93</v>
+      </c>
+      <c r="C95">
+        <v>2</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H95" t="s">
+        <v>40</v>
+      </c>
+      <c r="I95" t="s">
+        <v>210</v>
+      </c>
+      <c r="J95" t="s">
+        <v>240</v>
+      </c>
+      <c r="K95" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A96" s="1">
+        <v>94</v>
+      </c>
+      <c r="C96">
+        <v>3</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="H96" t="s">
+        <v>40</v>
+      </c>
+      <c r="I96" t="s">
+        <v>210</v>
+      </c>
+      <c r="J96" t="s">
+        <v>240</v>
+      </c>
+      <c r="K96" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A97" s="1">
+        <v>95</v>
+      </c>
+      <c r="C97">
+        <v>5</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="H97" t="s">
+        <v>40</v>
+      </c>
+      <c r="J97" t="s">
+        <v>240</v>
+      </c>
+      <c r="K97" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A98" s="1">
+        <v>96</v>
+      </c>
+      <c r="C98">
+        <v>5</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="H98" t="s">
+        <v>40</v>
+      </c>
+      <c r="I98" t="s">
+        <v>9</v>
+      </c>
+      <c r="J98" t="s">
+        <v>240</v>
+      </c>
+      <c r="K98" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A99" s="1">
+        <v>97</v>
+      </c>
+      <c r="C99">
+        <v>7</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="H99" t="s">
+        <v>40</v>
+      </c>
+      <c r="I99" t="s">
+        <v>9</v>
+      </c>
+      <c r="J99" t="s">
+        <v>240</v>
+      </c>
+      <c r="K99" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A100" s="1">
+        <v>98</v>
+      </c>
+      <c r="C100">
+        <v>0</v>
+      </c>
+      <c r="G100" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="H100" t="s">
+        <v>40</v>
+      </c>
+      <c r="I100" t="s">
+        <v>9</v>
+      </c>
+      <c r="J100" t="s">
+        <v>249</v>
+      </c>
+      <c r="K100" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A101" s="1">
+        <v>99</v>
+      </c>
+      <c r="C101">
+        <v>0</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="H101" t="s">
+        <v>40</v>
+      </c>
+      <c r="I101" t="s">
+        <v>9</v>
+      </c>
+      <c r="J101" t="s">
+        <v>249</v>
+      </c>
+      <c r="K101" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A102" s="1">
+        <v>100</v>
+      </c>
+      <c r="C102">
+        <v>1</v>
+      </c>
+      <c r="G102" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H102" t="s">
+        <v>40</v>
+      </c>
+      <c r="I102" t="s">
+        <v>9</v>
+      </c>
+      <c r="J102" t="s">
+        <v>249</v>
+      </c>
+      <c r="K102" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A103" s="1">
+        <v>101</v>
+      </c>
+      <c r="C103">
+        <v>1</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="H103" t="s">
+        <v>40</v>
+      </c>
+      <c r="I103" t="s">
+        <v>9</v>
+      </c>
+      <c r="J103" t="s">
+        <v>249</v>
+      </c>
+      <c r="K103" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A104" s="1">
+        <v>102</v>
+      </c>
+      <c r="C104">
+        <v>2</v>
+      </c>
+      <c r="G104" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="H104" t="s">
+        <v>40</v>
+      </c>
+      <c r="I104" t="s">
+        <v>254</v>
+      </c>
+      <c r="J104" t="s">
+        <v>249</v>
+      </c>
+      <c r="K104" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A105" s="1">
+        <v>103</v>
+      </c>
+      <c r="C105">
+        <v>2</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="H105" t="s">
+        <v>40</v>
+      </c>
+      <c r="I105" t="s">
+        <v>9</v>
+      </c>
+      <c r="J105" t="s">
+        <v>259</v>
+      </c>
+      <c r="K105" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A106" s="1">
+        <v>104</v>
+      </c>
+      <c r="C106">
+        <v>3</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="H106" t="s">
+        <v>40</v>
+      </c>
+      <c r="I106" t="s">
+        <v>210</v>
+      </c>
+      <c r="J106" t="s">
+        <v>249</v>
+      </c>
+      <c r="K106" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A107" s="1">
+        <v>105</v>
+      </c>
+      <c r="C107">
+        <v>4</v>
+      </c>
+      <c r="G107" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="H107" t="s">
+        <v>40</v>
+      </c>
+      <c r="I107" t="s">
+        <v>8</v>
+      </c>
+      <c r="J107" t="s">
+        <v>249</v>
+      </c>
+      <c r="K107" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A108" s="1">
+        <v>106</v>
+      </c>
+      <c r="C108">
+        <v>5</v>
+      </c>
+      <c r="G108" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="H108" t="s">
+        <v>40</v>
+      </c>
+      <c r="I108" t="s">
+        <v>9</v>
+      </c>
+      <c r="J108" t="s">
+        <v>249</v>
+      </c>
+      <c r="K108" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A109" s="1">
+        <v>107</v>
+      </c>
+      <c r="C109">
+        <v>6</v>
+      </c>
+      <c r="D109">
+        <v>6</v>
+      </c>
+      <c r="E109">
+        <v>5</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="H109" t="s">
+        <v>40</v>
+      </c>
+      <c r="I109" t="s">
+        <v>8</v>
+      </c>
+      <c r="J109" t="s">
+        <v>249</v>
+      </c>
+      <c r="K109" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A110" s="1">
+        <v>108</v>
+      </c>
+      <c r="C110">
+        <v>0</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H110" t="s">
+        <v>40</v>
+      </c>
+      <c r="I110" t="s">
+        <v>9</v>
+      </c>
+      <c r="J110" t="s">
+        <v>262</v>
+      </c>
+      <c r="K110" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A111" s="1">
+        <v>109</v>
+      </c>
+      <c r="C111">
+        <v>1</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="H111" t="s">
+        <v>40</v>
+      </c>
+      <c r="I111" t="s">
+        <v>210</v>
+      </c>
+      <c r="J111" t="s">
+        <v>262</v>
+      </c>
+      <c r="K111" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A112" s="1">
+        <v>110</v>
+      </c>
+      <c r="C112">
+        <v>1</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="H112" t="s">
+        <v>40</v>
+      </c>
+      <c r="I112" t="s">
+        <v>9</v>
+      </c>
+      <c r="J112" t="s">
+        <v>262</v>
+      </c>
+      <c r="K112" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A113" s="1">
+        <v>111</v>
+      </c>
+      <c r="C113">
+        <v>1</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="H113" t="s">
+        <v>40</v>
+      </c>
+      <c r="I113" t="s">
+        <v>210</v>
+      </c>
+      <c r="J113" t="s">
+        <v>262</v>
+      </c>
+      <c r="K113" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A114" s="1">
+        <v>112</v>
+      </c>
+      <c r="C114">
+        <v>1</v>
+      </c>
+      <c r="D114">
+        <v>1</v>
+      </c>
+      <c r="E114">
+        <v>3</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="H114" t="s">
+        <v>40</v>
+      </c>
+      <c r="I114" t="s">
+        <v>8</v>
+      </c>
+      <c r="J114" t="s">
+        <v>262</v>
+      </c>
+      <c r="K114" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A115" s="1">
+        <v>113</v>
+      </c>
+      <c r="C115">
+        <v>2</v>
+      </c>
+      <c r="D115">
+        <v>4</v>
+      </c>
+      <c r="E115">
+        <v>3</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="H115" t="s">
+        <v>40</v>
+      </c>
+      <c r="I115" t="s">
+        <v>8</v>
+      </c>
+      <c r="J115" t="s">
+        <v>262</v>
+      </c>
+      <c r="K115" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A116" s="1">
+        <v>114</v>
+      </c>
+      <c r="C116">
+        <v>3</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="H116" t="s">
+        <v>40</v>
+      </c>
+      <c r="I116" t="s">
+        <v>9</v>
+      </c>
+      <c r="J116" t="s">
+        <v>262</v>
+      </c>
+      <c r="K116" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A117" s="1">
+        <v>115</v>
+      </c>
+      <c r="C117">
+        <v>3</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="H117" t="s">
+        <v>40</v>
+      </c>
+      <c r="I117" t="s">
+        <v>9</v>
+      </c>
+      <c r="J117" t="s">
+        <v>262</v>
+      </c>
+      <c r="K117" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A118" s="1">
+        <v>116</v>
+      </c>
+      <c r="C118">
+        <v>4</v>
+      </c>
+      <c r="G118" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="H118" t="s">
+        <v>40</v>
+      </c>
+      <c r="I118" t="s">
+        <v>9</v>
+      </c>
+      <c r="J118" t="s">
+        <v>262</v>
+      </c>
+      <c r="K118" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A119" s="1">
+        <v>117</v>
+      </c>
+      <c r="C119">
+        <v>6</v>
+      </c>
+      <c r="D119">
+        <v>6</v>
+      </c>
+      <c r="E119">
+        <v>6</v>
+      </c>
+      <c r="G119" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="H119" t="s">
+        <v>40</v>
+      </c>
+      <c r="I119" t="s">
+        <v>8</v>
+      </c>
+      <c r="J119" t="s">
+        <v>262</v>
+      </c>
+      <c r="K119" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A120" s="1">
+        <v>118</v>
+      </c>
+      <c r="C120">
+        <v>1</v>
+      </c>
+      <c r="G120" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="H120" t="s">
+        <v>40</v>
+      </c>
+      <c r="I120" t="s">
+        <v>9</v>
+      </c>
+      <c r="J120" t="s">
+        <v>274</v>
+      </c>
+      <c r="K120" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A121" s="1">
+        <v>119</v>
+      </c>
+      <c r="C121">
+        <v>1</v>
+      </c>
+      <c r="G121" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="H121" t="s">
+        <v>40</v>
+      </c>
+      <c r="I121" t="s">
+        <v>9</v>
+      </c>
+      <c r="J121" t="s">
+        <v>273</v>
+      </c>
+      <c r="K121" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A122" s="1">
+        <v>120</v>
+      </c>
+      <c r="C122">
+        <v>2</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="H122" t="s">
+        <v>40</v>
+      </c>
+      <c r="I122" t="s">
+        <v>210</v>
+      </c>
+      <c r="J122" t="s">
+        <v>273</v>
+      </c>
+      <c r="K122" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A123" s="1">
+        <v>121</v>
+      </c>
+      <c r="C123">
+        <v>2</v>
+      </c>
+      <c r="G123" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="H123" t="s">
+        <v>40</v>
+      </c>
+      <c r="I123" t="s">
+        <v>210</v>
+      </c>
+      <c r="J123" t="s">
+        <v>273</v>
+      </c>
+      <c r="K123" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A124" s="1">
+        <v>122</v>
+      </c>
+      <c r="C124">
+        <v>2</v>
+      </c>
+      <c r="G124" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="H124" t="s">
+        <v>40</v>
+      </c>
+      <c r="I124" t="s">
+        <v>9</v>
+      </c>
+      <c r="J124" t="s">
+        <v>273</v>
+      </c>
+      <c r="K124" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A125" s="1">
+        <v>123</v>
+      </c>
+      <c r="C125">
+        <v>2</v>
+      </c>
+      <c r="G125" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="H125" t="s">
+        <v>40</v>
+      </c>
+      <c r="I125" t="s">
+        <v>9</v>
+      </c>
+      <c r="J125" t="s">
+        <v>273</v>
+      </c>
+      <c r="K125" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A126" s="1">
+        <v>124</v>
+      </c>
+      <c r="C126">
+        <v>3</v>
+      </c>
+      <c r="G126" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="H126" t="s">
+        <v>40</v>
+      </c>
+      <c r="I126" t="s">
+        <v>9</v>
+      </c>
+      <c r="J126" t="s">
+        <v>273</v>
+      </c>
+      <c r="K126" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A127" s="1">
+        <v>125</v>
+      </c>
+      <c r="C127">
+        <v>3</v>
+      </c>
+      <c r="D127">
+        <v>2</v>
+      </c>
+      <c r="E127">
+        <v>3</v>
+      </c>
+      <c r="G127" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="H127" t="s">
+        <v>40</v>
+      </c>
+      <c r="I127" t="s">
+        <v>8</v>
+      </c>
+      <c r="J127" t="s">
+        <v>273</v>
+      </c>
+      <c r="K127" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A128" s="1">
+        <v>126</v>
+      </c>
+      <c r="C128">
+        <v>4</v>
+      </c>
+      <c r="D128">
+        <v>4</v>
+      </c>
+      <c r="E128">
+        <v>3</v>
+      </c>
+      <c r="G128" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="H128" t="s">
+        <v>40</v>
+      </c>
+      <c r="I128" t="s">
+        <v>254</v>
+      </c>
+      <c r="J128" t="s">
+        <v>273</v>
+      </c>
+      <c r="K128" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A129" s="1">
+        <v>127</v>
+      </c>
+      <c r="C129">
+        <v>5</v>
+      </c>
+      <c r="G129" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="H129" t="s">
+        <v>40</v>
+      </c>
+      <c r="J129" t="s">
+        <v>273</v>
+      </c>
+      <c r="K129" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="6">
@@ -3589,7 +5427,7 @@
       <formula1>"자연,비전,화염,냉기,신성,암흑,None"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1:J1048576">
-      <formula1>"전사,사제,사냥꾼,드루이드,마법사,성기사,도적,주술사,중립"</formula1>
+      <formula1>"전사,사제,사냥꾼,드루이드,마법사,성기사,도적,주술사,중립,흑마법사"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1:L1048576">
       <formula1>"멀록,야수,None,정령,기계,용족"</formula1>

</xml_diff>